<commit_message>
Add a conf. paper.
</commit_message>
<xml_diff>
--- a/journal_pubs.xlsx
+++ b/journal_pubs.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Dropbox\Prof\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\crazytb\Code\curriculum_vitae\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{777BBE1A-075B-4A07-83B9-C695A814D1BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B68757F-3452-45AE-A65A-3D5904FC398F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="19110" yWindow="0" windowWidth="19380" windowHeight="20970" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="270">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="328" uniqueCount="274">
   <si>
     <t>ISSN</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -2453,6 +2453,22 @@
   </si>
   <si>
     <t>INSTRUMENTS &amp; INSTRUMENTATION</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Impact of Frame Duration on Cross-Channel Interference and Coexistence in IEEE 802.11bn NPCA</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Jisoo Lee and Taewon Song</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2025.10.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>2025 16th International Conference on Information and Communication Technology Convergence (ICTC)</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -2667,10 +2683,65 @@
         <sz val="10"/>
         <color auto="1"/>
         <name val="Myriad Pro"/>
-        <family val="2"/>
         <scheme val="none"/>
       </font>
-      <numFmt numFmtId="30" formatCode="@"/>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Myriad Pro"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Myriad Pro"/>
+        <scheme val="none"/>
+      </font>
+      <numFmt numFmtId="177" formatCode="0.0_);[Red]\(0.0\)"/>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color auto="1"/>
+        <name val="Myriad Pro"/>
+        <scheme val="none"/>
+      </font>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -2709,7 +2780,7 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
-      <numFmt numFmtId="177" formatCode="0.0_);[Red]\(0.0\)"/>
+      <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -2729,7 +2800,7 @@
         <family val="2"/>
         <scheme val="none"/>
       </font>
-      <numFmt numFmtId="30" formatCode="@"/>
+      <numFmt numFmtId="177" formatCode="0.0_);[Red]\(0.0\)"/>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -2765,65 +2836,10 @@
         <sz val="10"/>
         <color auto="1"/>
         <name val="Myriad Pro"/>
+        <family val="2"/>
         <scheme val="none"/>
       </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Myriad Pro"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Myriad Pro"/>
-        <scheme val="none"/>
-      </font>
-      <numFmt numFmtId="177" formatCode="0.0_);[Red]\(0.0\)"/>
-      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="10"/>
-        <color auto="1"/>
-        <name val="Myriad Pro"/>
-        <scheme val="none"/>
-      </font>
+      <numFmt numFmtId="30" formatCode="@"/>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
@@ -3101,17 +3117,17 @@
     <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="ISSN" dataDxfId="11"/>
     <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="권호 (Vol, Issue)" dataDxfId="10"/>
     <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="페이지" dataDxfId="9"/>
-    <tableColumn id="20" xr3:uid="{E8567B7E-7615-48B2-A9F1-1ECB9ED0DFE1}" name="분야" dataDxfId="0"/>
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Impact Factor" dataDxfId="4"/>
-    <tableColumn id="19" xr3:uid="{B70C4D17-BBEE-49CA-ADAC-A12EFA62BA3A}" name="JCR" dataDxfId="2" dataCellStyle="백분율"/>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Rating" dataDxfId="3"/>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="기본점수" dataDxfId="1" dataCellStyle="백분율"/>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="환산율" dataDxfId="8"/>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="가중치" dataDxfId="7" dataCellStyle="백분율"/>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="열3" dataDxfId="6">
+    <tableColumn id="20" xr3:uid="{E8567B7E-7615-48B2-A9F1-1ECB9ED0DFE1}" name="분야" dataDxfId="8"/>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Impact Factor" dataDxfId="7"/>
+    <tableColumn id="19" xr3:uid="{B70C4D17-BBEE-49CA-ADAC-A12EFA62BA3A}" name="JCR" dataDxfId="6" dataCellStyle="백분율"/>
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Rating" dataDxfId="5"/>
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="기본점수" dataDxfId="4" dataCellStyle="백분율"/>
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="환산율" dataDxfId="3"/>
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="가중치" dataDxfId="2" dataCellStyle="백분율"/>
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="열3" dataDxfId="1">
       <calculatedColumnFormula>표1[[#This Row],[환산율]]*표1[[#This Row],[가중치]]*표1[[#This Row],[기본점수]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="열4" dataDxfId="5">
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="열4" dataDxfId="0">
       <calculatedColumnFormula>SUM(표1[열3])</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -3314,7 +3330,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:U50"/>
+  <dimension ref="A1:U51"/>
   <sheetFormatPr defaultColWidth="8.6328125" defaultRowHeight="12.5"/>
   <cols>
     <col min="1" max="1" width="6.36328125" style="1" customWidth="1"/>
@@ -4432,22 +4448,22 @@
     </row>
     <row r="27" spans="1:21" ht="62.5">
       <c r="C27" s="1" t="s">
-        <v>246</v>
+        <v>270</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>243</v>
+        <v>271</v>
       </c>
       <c r="E27" s="1">
         <v>1</v>
       </c>
       <c r="F27" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G27" s="6" t="s">
-        <v>247</v>
+        <v>272</v>
       </c>
       <c r="H27" s="1" t="s">
-        <v>248</v>
+        <v>273</v>
       </c>
       <c r="I27" s="4" t="s">
         <v>105</v>
@@ -4455,22 +4471,22 @@
     </row>
     <row r="28" spans="1:21" ht="62.5">
       <c r="C28" s="1" t="s">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="E28" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F28" s="1">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G28" s="6" t="s">
-        <v>241</v>
+        <v>247</v>
       </c>
       <c r="H28" s="1" t="s">
-        <v>239</v>
+        <v>248</v>
       </c>
       <c r="I28" s="4" t="s">
         <v>105</v>
@@ -4478,16 +4494,16 @@
     </row>
     <row r="29" spans="1:21" ht="62.5">
       <c r="C29" s="1" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="E29" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F29" s="1">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G29" s="6" t="s">
         <v>241</v>
@@ -4501,16 +4517,16 @@
     </row>
     <row r="30" spans="1:21" ht="62.5">
       <c r="C30" s="1" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="E30" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F30" s="1">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G30" s="6" t="s">
         <v>241</v>
@@ -4522,81 +4538,81 @@
         <v>105</v>
       </c>
     </row>
-    <row r="31" spans="1:21" ht="50">
+    <row r="31" spans="1:21" ht="62.5">
       <c r="C31" s="1" t="s">
-        <v>51</v>
+        <v>238</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>52</v>
+        <v>240</v>
       </c>
       <c r="E31" s="1">
         <v>0</v>
       </c>
       <c r="F31" s="1">
+        <v>3</v>
+      </c>
+      <c r="G31" s="6" t="s">
+        <v>241</v>
+      </c>
+      <c r="H31" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="I31" s="4" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="32" spans="1:21" ht="50">
+      <c r="C32" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="E32" s="1">
+        <v>0</v>
+      </c>
+      <c r="F32" s="1">
         <v>4</v>
       </c>
-      <c r="G31" s="6" t="s">
+      <c r="G32" s="6" t="s">
         <v>53</v>
       </c>
-      <c r="H31" s="1" t="s">
+      <c r="H32" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="I31" s="4" t="s">
+      <c r="I32" s="4" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="32" spans="1:21" ht="37.5">
-      <c r="C32" s="1" t="s">
+    <row r="33" spans="3:11" ht="37.5">
+      <c r="C33" s="1" t="s">
         <v>170</v>
       </c>
-      <c r="D32" s="1" t="s">
+      <c r="D33" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="E32" s="1">
+      <c r="E33" s="1">
         <v>1</v>
       </c>
-      <c r="F32" s="1">
+      <c r="F33" s="1">
         <v>2</v>
       </c>
-      <c r="G32" s="6" t="s">
+      <c r="G33" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="H32" s="1" t="s">
+      <c r="H33" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="I32" s="4" t="s">
+      <c r="I33" s="4" t="s">
         <v>105</v>
-      </c>
-    </row>
-    <row r="33" spans="3:11" ht="62.5">
-      <c r="C33" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="D33" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="E33" s="1">
-        <v>0</v>
-      </c>
-      <c r="F33" s="1">
-        <v>4</v>
-      </c>
-      <c r="G33" s="6" t="s">
-        <v>60</v>
-      </c>
-      <c r="H33" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="I33" s="4" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="34" spans="3:11" ht="62.5">
       <c r="C34" s="1" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="E34" s="1">
         <v>0</v>
@@ -4605,7 +4621,7 @@
         <v>4</v>
       </c>
       <c r="G34" s="6" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="H34" s="1" t="s">
         <v>136</v>
@@ -4614,15 +4630,15 @@
         <v>106</v>
       </c>
     </row>
-    <row r="35" spans="3:11" ht="37.5">
+    <row r="35" spans="3:11" ht="62.5">
       <c r="C35" s="1" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="E35" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F35" s="1">
         <v>4</v>
@@ -4631,194 +4647,188 @@
         <v>63</v>
       </c>
       <c r="H35" s="1" t="s">
-        <v>66</v>
+        <v>136</v>
       </c>
       <c r="I35" s="4" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="36" spans="3:11" ht="37.5">
       <c r="C36" s="1" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="E36" s="1">
         <v>1</v>
       </c>
       <c r="F36" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G36" s="6" t="s">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="H36" s="1" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="I36" s="4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
-    <row r="37" spans="3:11" ht="25">
+    <row r="37" spans="3:11" ht="37.5">
       <c r="C37" s="1" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="E37" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F37" s="1">
         <v>3</v>
       </c>
       <c r="G37" s="6" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="H37" s="1" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="I37" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
-    <row r="38" spans="3:11" ht="37.5">
+    <row r="38" spans="3:11" ht="25">
       <c r="C38" s="1" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="E38" s="1">
         <v>0</v>
       </c>
       <c r="F38" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G38" s="6" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="H38" s="1" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="I38" s="4" t="s">
-        <v>171</v>
+        <v>109</v>
       </c>
     </row>
     <row r="39" spans="3:11" ht="37.5">
       <c r="C39" s="1" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="E39" s="1">
         <v>0</v>
       </c>
       <c r="F39" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G39" s="6" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="H39" s="1" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="I39" s="4" t="s">
-        <v>110</v>
+        <v>171</v>
       </c>
     </row>
-    <row r="40" spans="3:11" ht="62.5">
+    <row r="40" spans="3:11" ht="37.5">
       <c r="C40" s="1" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="E40" s="1">
         <v>0</v>
       </c>
       <c r="F40" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G40" s="6" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="H40" s="1" t="s">
-        <v>137</v>
+        <v>82</v>
       </c>
       <c r="I40" s="4" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="41" spans="3:11" ht="62.5">
       <c r="C41" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="D41" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="E41" s="1">
+        <v>0</v>
+      </c>
+      <c r="F41" s="1">
+        <v>4</v>
+      </c>
+      <c r="G41" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="H41" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="I41" s="4" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="42" spans="3:11" ht="62.5">
+      <c r="C42" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="D41" s="1" t="s">
+      <c r="D42" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="E41" s="1">
+      <c r="E42" s="1">
         <v>1</v>
       </c>
-      <c r="F41" s="1">
+      <c r="F42" s="1">
         <v>3</v>
       </c>
-      <c r="G41" s="6" t="s">
+      <c r="G42" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="H41" s="1" t="s">
+      <c r="H42" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="I41" s="4" t="s">
+      <c r="I42" s="4" t="s">
         <v>110</v>
-      </c>
-    </row>
-    <row r="42" spans="3:11" ht="26">
-      <c r="C42" s="1" t="s">
-        <v>149</v>
-      </c>
-      <c r="D42" s="1" t="s">
-        <v>150</v>
-      </c>
-      <c r="E42" s="1">
-        <v>0</v>
-      </c>
-      <c r="F42" s="1">
-        <v>4</v>
-      </c>
-      <c r="G42" s="6" t="s">
-        <v>117</v>
-      </c>
-      <c r="H42" s="1" t="s">
-        <v>151</v>
-      </c>
-      <c r="I42" s="4" t="s">
-        <v>112</v>
-      </c>
-      <c r="J42" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="K42" s="4" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="43" spans="3:11" ht="26">
       <c r="C43" s="1" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="E43" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F43" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G43" s="6" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="H43" s="1" t="s">
         <v>151</v>
@@ -4827,27 +4837,27 @@
         <v>112</v>
       </c>
       <c r="J43" s="4" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="K43" s="4" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
-    <row r="44" spans="3:11" ht="39">
+    <row r="44" spans="3:11" ht="26">
       <c r="C44" s="1" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="E44" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F44" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G44" s="6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="H44" s="1" t="s">
         <v>151</v>
@@ -4856,18 +4866,18 @@
         <v>112</v>
       </c>
       <c r="J44" s="4" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="K44" s="4" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
-    <row r="45" spans="3:11" ht="26">
+    <row r="45" spans="3:11" ht="39">
       <c r="C45" s="1" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="E45" s="1">
         <v>0</v>
@@ -4876,87 +4886,116 @@
         <v>4</v>
       </c>
       <c r="G45" s="6" t="s">
-        <v>96</v>
+        <v>119</v>
       </c>
       <c r="H45" s="1" t="s">
-        <v>158</v>
+        <v>151</v>
       </c>
       <c r="I45" s="4" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="J45" s="4" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="K45" s="4" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="46" spans="3:11" ht="26">
       <c r="C46" s="1" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="E46" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F46" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G46" s="6" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="H46" s="1" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="I46" s="4" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="J46" s="4" t="s">
-        <v>115</v>
+        <v>97</v>
       </c>
       <c r="K46" s="4" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="47" spans="3:11" ht="26">
       <c r="C47" s="1" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="E47" s="1">
         <v>1</v>
       </c>
       <c r="F47" s="1">
+        <v>2</v>
+      </c>
+      <c r="G47" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="H47" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="I47" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="J47" s="4" t="s">
+        <v>115</v>
+      </c>
+      <c r="K47" s="4" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="48" spans="3:11" ht="26">
+      <c r="C48" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="D48" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="E48" s="1">
+        <v>1</v>
+      </c>
+      <c r="F48" s="1">
         <v>4</v>
       </c>
-      <c r="G47" s="6" t="s">
+      <c r="G48" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="H47" s="1" t="s">
+      <c r="H48" s="1" t="s">
         <v>164</v>
       </c>
-      <c r="I47" s="4" t="s">
+      <c r="I48" s="4" t="s">
         <v>116</v>
       </c>
-      <c r="J47" s="4" t="s">
+      <c r="J48" s="4" t="s">
         <v>102</v>
       </c>
-      <c r="K47" s="4" t="s">
+      <c r="K48" s="4" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="50" spans="1:7" ht="48">
-      <c r="A50" s="1" t="s">
+    <row r="51" spans="1:7" ht="48">
+      <c r="A51" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C50" s="1" t="s">
+      <c r="C51" s="1" t="s">
         <v>131</v>
       </c>
-      <c r="G50" s="6" t="s">
+      <c r="G51" s="6" t="s">
         <v>22</v>
       </c>
     </row>

</xml_diff>